<commit_message>
Actualización automática: datos al 2026-06-27
</commit_message>
<xml_diff>
--- a/atlantida.xlsx
+++ b/atlantida.xlsx
@@ -1595,7 +1595,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-26)</t>
+          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-27)</t>
         </is>
       </c>
     </row>
@@ -4266,7 +4266,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-26) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-27) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4427,7 +4427,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-26)</t>
+          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-27)</t>
         </is>
       </c>
     </row>
@@ -6342,7 +6342,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-26) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-27) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -78578,7 +78578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-26)</t>
+          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-27)</t>
         </is>
       </c>
     </row>
@@ -79968,7 +79968,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-26)</t>
+          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-27)</t>
         </is>
       </c>
     </row>
@@ -81267,7 +81267,7 @@
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>datos al 2026-06-27 (actualización 2026-06-26).</t>
+          <t>datos al 2026-06-27 (actualización 2026-06-27).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-06-28
</commit_message>
<xml_diff>
--- a/atlantida.xlsx
+++ b/atlantida.xlsx
@@ -1595,7 +1595,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-27)</t>
+          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-28)</t>
         </is>
       </c>
     </row>
@@ -4266,7 +4266,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-27) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-28) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4427,7 +4427,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-27)</t>
+          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-28)</t>
         </is>
       </c>
     </row>
@@ -6342,7 +6342,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-27) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-28) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -78578,7 +78578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-27)</t>
+          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-28)</t>
         </is>
       </c>
     </row>
@@ -79968,7 +79968,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-27)</t>
+          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-28)</t>
         </is>
       </c>
     </row>
@@ -81267,7 +81267,7 @@
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>datos al 2026-06-27 (actualización 2026-06-27).</t>
+          <t>datos al 2026-06-27 (actualización 2026-06-28).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-06-29
</commit_message>
<xml_diff>
--- a/atlantida.xlsx
+++ b/atlantida.xlsx
@@ -1595,7 +1595,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-28)</t>
+          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-29)</t>
         </is>
       </c>
     </row>
@@ -4266,7 +4266,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-28) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-29) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4427,7 +4427,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-28)</t>
+          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-29)</t>
         </is>
       </c>
     </row>
@@ -6342,7 +6342,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-28) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-29) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -78578,7 +78578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-28)</t>
+          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-29)</t>
         </is>
       </c>
     </row>
@@ -79968,7 +79968,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-28)</t>
+          <t>Atlántida Capital | Fuente: atlantidacapital.com.sv | datos al 2026-06-27 (actualización 2026-06-29)</t>
         </is>
       </c>
     </row>
@@ -81267,7 +81267,7 @@
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>datos al 2026-06-27 (actualización 2026-06-28).</t>
+          <t>datos al 2026-06-27 (actualización 2026-06-29).</t>
         </is>
       </c>
     </row>

</xml_diff>